<commit_message>
update few shot examples
</commit_message>
<xml_diff>
--- a/data/describe/few_shot/few_shot_examples.xlsx
+++ b/data/describe/few_shot/few_shot_examples.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\few_shot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECE76857-E38D-49D5-AB16-A042A12AAF91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C8724AA-3D3F-4A88-83DB-D3A39AA788EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="55260" yWindow="1620" windowWidth="22410" windowHeight="15465" xr2:uid="{16C02B7C-A662-4920-9F10-20A7161C31E3}"/>
+    <workbookView xWindow="51150" yWindow="1305" windowWidth="27195" windowHeight="17070" xr2:uid="{16C02B7C-A662-4920-9F10-20A7161C31E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>